<commit_message>
Initial commit on v2 branch
</commit_message>
<xml_diff>
--- a/data/draw_history.xlsx
+++ b/data/draw_history.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MacMiniExt/Personal/Lotto/lotto_predictor/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/MacMiniExt/Personal/Lotto/lotto_predictor_v2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7859CF42-34C4-2443-9709-99FE8B291E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35619CCD-37EC-3C40-99A5-30503550EE55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57740" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2100" yWindow="2280" windowWidth="51200" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet5" sheetId="1" r:id="rId1"/>
@@ -50648,159 +50648,411 @@
       <c r="J1677" s="4"/>
     </row>
     <row r="1678" spans="1:10" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1678" s="3"/>
-      <c r="B1678" s="4"/>
-      <c r="C1678" s="4"/>
-      <c r="D1678" s="4"/>
-      <c r="E1678" s="4"/>
-      <c r="F1678" s="4"/>
-      <c r="G1678" s="4"/>
-      <c r="H1678" s="4"/>
-      <c r="I1678" s="4"/>
+      <c r="A1678" s="3">
+        <v>2477</v>
+      </c>
+      <c r="B1678" s="5">
+        <v>45777</v>
+      </c>
+      <c r="C1678" s="3">
+        <v>1</v>
+      </c>
+      <c r="D1678" s="3">
+        <v>12</v>
+      </c>
+      <c r="E1678" s="3">
+        <v>14</v>
+      </c>
+      <c r="F1678" s="3">
+        <v>20</v>
+      </c>
+      <c r="G1678" s="3">
+        <v>24</v>
+      </c>
+      <c r="H1678" s="3">
+        <v>38</v>
+      </c>
+      <c r="I1678" s="3">
+        <v>4</v>
+      </c>
       <c r="J1678" s="4"/>
     </row>
     <row r="1679" spans="1:10" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1679" s="1"/>
-      <c r="B1679" s="2"/>
-      <c r="C1679" s="1"/>
-      <c r="D1679" s="1"/>
-      <c r="E1679" s="1"/>
-      <c r="F1679" s="1"/>
-      <c r="G1679" s="1"/>
-      <c r="H1679" s="1"/>
-      <c r="I1679" s="1"/>
+      <c r="A1679" s="3">
+        <v>2478</v>
+      </c>
+      <c r="B1679" s="5">
+        <v>45780</v>
+      </c>
+      <c r="C1679" s="3">
+        <v>1</v>
+      </c>
+      <c r="D1679" s="3">
+        <v>11</v>
+      </c>
+      <c r="E1679" s="3">
+        <v>13</v>
+      </c>
+      <c r="F1679" s="3">
+        <v>21</v>
+      </c>
+      <c r="G1679" s="3">
+        <v>22</v>
+      </c>
+      <c r="H1679" s="3">
+        <v>23</v>
+      </c>
+      <c r="I1679" s="3">
+        <v>10</v>
+      </c>
     </row>
     <row r="1680" spans="1:10" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1680" s="1"/>
-      <c r="B1680" s="2"/>
-      <c r="C1680" s="1"/>
-      <c r="D1680" s="1"/>
-      <c r="E1680" s="1"/>
-      <c r="F1680" s="1"/>
-      <c r="G1680" s="1"/>
-      <c r="H1680" s="1"/>
-      <c r="I1680" s="1"/>
+      <c r="A1680" s="3">
+        <v>2479</v>
+      </c>
+      <c r="B1680" s="6">
+        <v>45784</v>
+      </c>
+      <c r="C1680" s="3">
+        <v>9</v>
+      </c>
+      <c r="D1680" s="3">
+        <v>11</v>
+      </c>
+      <c r="E1680" s="3">
+        <v>13</v>
+      </c>
+      <c r="F1680" s="3">
+        <v>18</v>
+      </c>
+      <c r="G1680" s="3">
+        <v>26</v>
+      </c>
+      <c r="H1680" s="3">
+        <v>36</v>
+      </c>
+      <c r="I1680" s="3">
+        <v>7</v>
+      </c>
     </row>
     <row r="1681" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1681" s="1"/>
-      <c r="B1681" s="2"/>
-      <c r="C1681" s="1"/>
-      <c r="D1681" s="1"/>
-      <c r="E1681" s="1"/>
-      <c r="F1681" s="1"/>
-      <c r="G1681" s="1"/>
-      <c r="H1681" s="1"/>
-      <c r="I1681" s="1"/>
+      <c r="A1681" s="3">
+        <v>2480</v>
+      </c>
+      <c r="B1681" s="5">
+        <v>45787</v>
+      </c>
+      <c r="C1681" s="3">
+        <v>4</v>
+      </c>
+      <c r="D1681" s="3">
+        <v>14</v>
+      </c>
+      <c r="E1681" s="3">
+        <v>17</v>
+      </c>
+      <c r="F1681" s="3">
+        <v>22</v>
+      </c>
+      <c r="G1681" s="3">
+        <v>27</v>
+      </c>
+      <c r="H1681" s="3">
+        <v>35</v>
+      </c>
+      <c r="I1681" s="3">
+        <v>6</v>
+      </c>
     </row>
     <row r="1682" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1682" s="1"/>
-      <c r="B1682" s="2"/>
-      <c r="C1682" s="1"/>
-      <c r="D1682" s="1"/>
-      <c r="E1682" s="1"/>
-      <c r="F1682" s="1"/>
-      <c r="G1682" s="1"/>
-      <c r="H1682" s="1"/>
-      <c r="I1682" s="1"/>
+      <c r="A1682" s="3">
+        <v>2481</v>
+      </c>
+      <c r="B1682" s="5">
+        <v>45791</v>
+      </c>
+      <c r="C1682" s="3">
+        <v>1</v>
+      </c>
+      <c r="D1682" s="3">
+        <v>6</v>
+      </c>
+      <c r="E1682" s="3">
+        <v>8</v>
+      </c>
+      <c r="F1682" s="3">
+        <v>21</v>
+      </c>
+      <c r="G1682" s="3">
+        <v>27</v>
+      </c>
+      <c r="H1682" s="3">
+        <v>28</v>
+      </c>
+      <c r="I1682" s="3">
+        <v>9</v>
+      </c>
     </row>
     <row r="1683" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1683" s="1"/>
-      <c r="B1683" s="2"/>
-      <c r="C1683" s="1"/>
-      <c r="D1683" s="1"/>
-      <c r="E1683" s="1"/>
-      <c r="F1683" s="1"/>
-      <c r="G1683" s="1"/>
-      <c r="H1683" s="1"/>
-      <c r="I1683" s="1"/>
+      <c r="A1683" s="3">
+        <v>2482</v>
+      </c>
+      <c r="B1683" s="6">
+        <v>45794</v>
+      </c>
+      <c r="C1683" s="3">
+        <v>2</v>
+      </c>
+      <c r="D1683" s="3">
+        <v>6</v>
+      </c>
+      <c r="E1683" s="3">
+        <v>15</v>
+      </c>
+      <c r="F1683" s="3">
+        <v>19</v>
+      </c>
+      <c r="G1683" s="3">
+        <v>22</v>
+      </c>
+      <c r="H1683" s="3">
+        <v>25</v>
+      </c>
+      <c r="I1683" s="3">
+        <v>7</v>
+      </c>
     </row>
     <row r="1684" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1684" s="1"/>
-      <c r="B1684" s="2"/>
-      <c r="C1684" s="1"/>
-      <c r="D1684" s="1"/>
-      <c r="E1684" s="1"/>
-      <c r="F1684" s="1"/>
-      <c r="G1684" s="1"/>
-      <c r="H1684" s="1"/>
-      <c r="I1684" s="1"/>
+      <c r="A1684" s="3">
+        <v>2483</v>
+      </c>
+      <c r="B1684" s="5">
+        <v>45798</v>
+      </c>
+      <c r="C1684" s="3">
+        <v>3</v>
+      </c>
+      <c r="D1684" s="3">
+        <v>5</v>
+      </c>
+      <c r="E1684" s="3">
+        <v>6</v>
+      </c>
+      <c r="F1684" s="3">
+        <v>24</v>
+      </c>
+      <c r="G1684" s="3">
+        <v>27</v>
+      </c>
+      <c r="H1684" s="3">
+        <v>37</v>
+      </c>
+      <c r="I1684" s="3">
+        <v>10</v>
+      </c>
     </row>
     <row r="1685" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1685" s="1"/>
-      <c r="B1685" s="2"/>
-      <c r="C1685" s="1"/>
-      <c r="D1685" s="1"/>
-      <c r="E1685" s="1"/>
-      <c r="F1685" s="1"/>
-      <c r="G1685" s="1"/>
-      <c r="H1685" s="1"/>
-      <c r="I1685" s="1"/>
+      <c r="A1685" s="3">
+        <v>2484</v>
+      </c>
+      <c r="B1685" s="5">
+        <v>45801</v>
+      </c>
+      <c r="C1685" s="3">
+        <v>1</v>
+      </c>
+      <c r="D1685" s="3">
+        <v>7</v>
+      </c>
+      <c r="E1685" s="3">
+        <v>27</v>
+      </c>
+      <c r="F1685" s="3">
+        <v>29</v>
+      </c>
+      <c r="G1685" s="3">
+        <v>36</v>
+      </c>
+      <c r="H1685" s="3">
+        <v>38</v>
+      </c>
+      <c r="I1685" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="1686" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1686" s="1"/>
-      <c r="B1686" s="2"/>
-      <c r="C1686" s="1"/>
-      <c r="D1686" s="1"/>
-      <c r="E1686" s="1"/>
-      <c r="F1686" s="1"/>
-      <c r="G1686" s="1"/>
-      <c r="H1686" s="1"/>
-      <c r="I1686" s="1"/>
+      <c r="A1686" s="3">
+        <v>2485</v>
+      </c>
+      <c r="B1686" s="6">
+        <v>45805</v>
+      </c>
+      <c r="C1686" s="3">
+        <v>1</v>
+      </c>
+      <c r="D1686" s="3">
+        <v>10</v>
+      </c>
+      <c r="E1686" s="3">
+        <v>15</v>
+      </c>
+      <c r="F1686" s="3">
+        <v>18</v>
+      </c>
+      <c r="G1686" s="3">
+        <v>25</v>
+      </c>
+      <c r="H1686" s="3">
+        <v>40</v>
+      </c>
+      <c r="I1686" s="3">
+        <v>7</v>
+      </c>
     </row>
     <row r="1687" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1687" s="1"/>
-      <c r="B1687" s="2"/>
-      <c r="C1687" s="1"/>
-      <c r="D1687" s="1"/>
-      <c r="E1687" s="1"/>
-      <c r="F1687" s="1"/>
-      <c r="G1687" s="1"/>
-      <c r="H1687" s="1"/>
-      <c r="I1687" s="1"/>
+      <c r="A1687" s="3">
+        <v>2486</v>
+      </c>
+      <c r="B1687" s="5">
+        <v>45808</v>
+      </c>
+      <c r="C1687" s="3">
+        <v>1</v>
+      </c>
+      <c r="D1687" s="3">
+        <v>2</v>
+      </c>
+      <c r="E1687" s="3">
+        <v>29</v>
+      </c>
+      <c r="F1687" s="3">
+        <v>32</v>
+      </c>
+      <c r="G1687" s="3">
+        <v>34</v>
+      </c>
+      <c r="H1687" s="3">
+        <v>35</v>
+      </c>
+      <c r="I1687" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="1688" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1688" s="1"/>
-      <c r="B1688" s="2"/>
-      <c r="C1688" s="1"/>
-      <c r="D1688" s="1"/>
-      <c r="E1688" s="1"/>
-      <c r="F1688" s="1"/>
-      <c r="G1688" s="1"/>
-      <c r="H1688" s="1"/>
-      <c r="I1688" s="1"/>
+      <c r="A1688" s="3">
+        <v>2487</v>
+      </c>
+      <c r="B1688" s="5">
+        <v>45812</v>
+      </c>
+      <c r="C1688" s="3">
+        <v>6</v>
+      </c>
+      <c r="D1688" s="3">
+        <v>9</v>
+      </c>
+      <c r="E1688" s="3">
+        <v>10</v>
+      </c>
+      <c r="F1688" s="3">
+        <v>11</v>
+      </c>
+      <c r="G1688" s="3">
+        <v>14</v>
+      </c>
+      <c r="H1688" s="3">
+        <v>35</v>
+      </c>
+      <c r="I1688" s="3">
+        <v>10</v>
+      </c>
     </row>
     <row r="1689" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1689" s="1"/>
-      <c r="B1689" s="2"/>
-      <c r="C1689" s="1"/>
-      <c r="D1689" s="1"/>
-      <c r="E1689" s="1"/>
-      <c r="F1689" s="1"/>
-      <c r="G1689" s="1"/>
-      <c r="H1689" s="1"/>
-      <c r="I1689" s="1"/>
+      <c r="A1689" s="3">
+        <v>2488</v>
+      </c>
+      <c r="B1689" s="5">
+        <v>45815</v>
+      </c>
+      <c r="C1689" s="3">
+        <v>2</v>
+      </c>
+      <c r="D1689" s="3">
+        <v>6</v>
+      </c>
+      <c r="E1689" s="3">
+        <v>11</v>
+      </c>
+      <c r="F1689" s="3">
+        <v>16</v>
+      </c>
+      <c r="G1689" s="3">
+        <v>22</v>
+      </c>
+      <c r="H1689" s="3">
+        <v>34</v>
+      </c>
+      <c r="I1689" s="3">
+        <v>4</v>
+      </c>
     </row>
     <row r="1690" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1690" s="1"/>
-      <c r="B1690" s="2"/>
-      <c r="C1690" s="1"/>
-      <c r="D1690" s="1"/>
-      <c r="E1690" s="1"/>
-      <c r="F1690" s="1"/>
-      <c r="G1690" s="1"/>
-      <c r="H1690" s="1"/>
-      <c r="I1690" s="1"/>
+      <c r="A1690" s="3">
+        <v>2489</v>
+      </c>
+      <c r="B1690" s="6">
+        <v>45819</v>
+      </c>
+      <c r="C1690" s="3">
+        <v>5</v>
+      </c>
+      <c r="D1690" s="3">
+        <v>9</v>
+      </c>
+      <c r="E1690" s="3">
+        <v>11</v>
+      </c>
+      <c r="F1690" s="3">
+        <v>16</v>
+      </c>
+      <c r="G1690" s="3">
+        <v>18</v>
+      </c>
+      <c r="H1690" s="3">
+        <v>32</v>
+      </c>
+      <c r="I1690" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="1691" spans="1:9" ht="14" x14ac:dyDescent="0.2">
-      <c r="A1691" s="1"/>
-      <c r="B1691" s="2"/>
-      <c r="C1691" s="1"/>
-      <c r="D1691" s="1"/>
-      <c r="E1691" s="1"/>
-      <c r="F1691" s="1"/>
-      <c r="G1691" s="1"/>
-      <c r="H1691" s="1"/>
-      <c r="I1691" s="1"/>
+      <c r="A1691" s="3">
+        <v>2490</v>
+      </c>
+      <c r="B1691" s="5">
+        <v>45822</v>
+      </c>
+      <c r="C1691" s="3">
+        <v>1</v>
+      </c>
+      <c r="D1691" s="3">
+        <v>2</v>
+      </c>
+      <c r="E1691" s="3">
+        <v>7</v>
+      </c>
+      <c r="F1691" s="3">
+        <v>13</v>
+      </c>
+      <c r="G1691" s="3">
+        <v>23</v>
+      </c>
+      <c r="H1691" s="3">
+        <v>34</v>
+      </c>
+      <c r="I1691" s="3">
+        <v>6</v>
+      </c>
     </row>
     <row r="1692" spans="1:9" ht="14" x14ac:dyDescent="0.2">
       <c r="A1692" s="1"/>
@@ -60912,11 +61164,12 @@
       <c r="I2610" s="1"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B1679:B2610">
+  <conditionalFormatting sqref="B1692:B2610">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(B1679))&gt;0</formula>
+      <formula>LEN(TRIM(B1692))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>